<commit_message>
Checkpoint before resampling-pipeline audit: rebuild + incident-response work through 2026-09-08g
Safety-net commit ahead of a planned holistic audit of resampling/ -
recurring bugs traced to pre-rebuild ad-hoc fixes and duplicated logic
drifting out of sync are still surfacing (most recently an incorrect
sampling frame sent out today that needs withdrawing). Captures the
2026-09-07/08 incident response and rebuild (assert_fresh gates,
default-direction fix, v6->v7 rollback, FACT/partner redraws, Dandume/
Faskari reinstatement) plus the daily partner-workbook refresh tier -
all already-completed, verified work per 1_sampling/CLAUDE.md.

Excludes resampling/input/partner_raw_comms/ (raw partner email
correspondence) from version control - this is a public repo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resampling/input/accessibility_reports_generated/ACF_accessibility_report.xlsx
+++ b/resampling/input/accessibility_reports_generated/ACF_accessibility_report.xlsx
@@ -836,14 +836,11 @@
           <t>Bodinga Tauma</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>2</v>
       </c>
@@ -853,13 +850,36 @@
       <c r="J2" t="n">
         <v>67</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" s="10" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O2" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -877,14 +897,11 @@
           <t>Sifawa Lukuyawa</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>3</v>
       </c>
@@ -894,13 +911,7 @@
       <c r="J3" t="n">
         <v>26</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" s="10" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -918,14 +929,11 @@
           <t>Kaura Miyo</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>6</v>
       </c>
@@ -935,13 +943,7 @@
       <c r="J4" t="n">
         <v>23</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" s="10" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -959,7 +961,6 @@
           <t>Dingyadi</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -984,13 +985,36 @@
       <c r="J5" t="n">
         <v>18</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" s="10" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1008,14 +1032,11 @@
           <t>Danchadi</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>1</v>
       </c>
@@ -1025,13 +1046,36 @@
       <c r="J6" t="n">
         <v>11</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" s="10" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1049,14 +1093,11 @@
           <t>Bagarawa</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>4</v>
       </c>
@@ -1066,13 +1107,36 @@
       <c r="J7" t="n">
         <v>9</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" s="10" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1090,14 +1154,11 @@
           <t>Kwacciyar Lalle</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>2</v>
       </c>
@@ -1107,13 +1168,7 @@
       <c r="J8" t="n">
         <v>8</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" s="10" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1131,14 +1186,11 @@
           <t>Takatuku Madorawa</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>4</v>
       </c>
@@ -1148,13 +1200,36 @@
       <c r="J9" t="n">
         <v>8</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" s="10" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1172,14 +1247,11 @@
           <t>Bangi Dabaga</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>2</v>
       </c>
@@ -1189,13 +1261,36 @@
       <c r="J10" t="n">
         <v>7</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" s="10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1213,14 +1308,11 @@
           <t>Tulluwa</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>5</v>
       </c>
@@ -1230,13 +1322,36 @@
       <c r="J11" t="n">
         <v>7</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" s="10" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1254,14 +1369,11 @@
           <t>Darhela Badau</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>1</v>
       </c>
@@ -1271,13 +1383,7 @@
       <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" s="10" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1295,14 +1401,11 @@
           <t>Kammata</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>1</v>
       </c>
@@ -1312,13 +1415,7 @@
       <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" s="10" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1336,14 +1433,11 @@
           <t>Kagara</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>1</v>
       </c>
@@ -1353,13 +1447,7 @@
       <c r="J14" t="n">
         <v>62</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" s="10" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1377,14 +1465,11 @@
           <t>Goronyo</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>3</v>
       </c>
@@ -1394,13 +1479,7 @@
       <c r="J15" t="n">
         <v>36</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" s="10" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1418,14 +1497,11 @@
           <t>Rimawa</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>4</v>
       </c>
@@ -1435,13 +1511,7 @@
       <c r="J16" t="n">
         <v>30</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" s="10" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1459,14 +1529,11 @@
           <t>Shinaka</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>0</v>
       </c>
@@ -1476,13 +1543,7 @@
       <c r="J17" t="n">
         <v>18</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" s="10" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1500,14 +1561,11 @@
           <t>Takakume</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>2</v>
       </c>
@@ -1517,13 +1575,7 @@
       <c r="J18" t="n">
         <v>11</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" s="10" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1541,14 +1593,11 @@
           <t>Sabon Gari Dole</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>3</v>
       </c>
@@ -1558,13 +1607,7 @@
       <c r="J19" t="n">
         <v>9</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" s="10" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1582,14 +1625,11 @@
           <t>Giyawa</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>2</v>
       </c>
@@ -1599,13 +1639,7 @@
       <c r="J20" t="n">
         <v>8</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" s="10" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1623,14 +1657,11 @@
           <t>Birjingo</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>2</v>
       </c>
@@ -1640,13 +1671,7 @@
       <c r="J21" t="n">
         <v>7</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" s="10" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1664,14 +1689,11 @@
           <t>Kojiyo</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>1</v>
       </c>
@@ -1681,13 +1703,7 @@
       <c r="J22" t="n">
         <v>6</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" s="10" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1705,14 +1721,11 @@
           <t>Kwakwazo</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>1</v>
       </c>
@@ -1722,13 +1735,7 @@
       <c r="J23" t="n">
         <v>6</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" s="10" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1746,7 +1753,6 @@
           <t>Tidibale</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1771,13 +1777,7 @@
       <c r="J24" t="n">
         <v>4</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" s="10" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1795,14 +1795,11 @@
           <t>Boyekai</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>1</v>
       </c>
@@ -1812,13 +1809,7 @@
       <c r="J25" t="n">
         <v>1</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" s="10" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1836,14 +1827,11 @@
           <t>Gwadabawa</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>3</v>
       </c>
@@ -1853,13 +1841,36 @@
       <c r="J26" t="n">
         <v>43</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" s="10" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1877,7 +1888,6 @@
           <t>Salame</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1902,13 +1912,36 @@
       <c r="J27" t="n">
         <v>39</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" s="10" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1926,7 +1959,6 @@
           <t>Darna Sabon Gari</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1951,13 +1983,7 @@
       <c r="J28" t="n">
         <v>18</v>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" s="10" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1975,7 +2001,6 @@
           <t>Asara</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2000,13 +2025,36 @@
       <c r="J29" t="n">
         <v>17</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" s="10" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2024,14 +2072,11 @@
           <t>Tambagarka</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
         <v>3</v>
       </c>
@@ -2041,13 +2086,36 @@
       <c r="J30" t="n">
         <v>16</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" s="10" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2065,7 +2133,6 @@
           <t>Atakwanyo</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2090,13 +2157,36 @@
       <c r="J31" t="n">
         <v>14</v>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" s="10" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O31" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2114,14 +2204,11 @@
           <t>Gigane</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
         <v>2</v>
       </c>
@@ -2131,13 +2218,36 @@
       <c r="J32" t="n">
         <v>12</v>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" s="10" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2155,14 +2265,11 @@
           <t>Chimola</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>3</v>
       </c>
@@ -2172,13 +2279,36 @@
       <c r="J33" t="n">
         <v>11</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" s="10" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O33" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2196,14 +2326,11 @@
           <t>Huchi</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
         <v>2</v>
       </c>
@@ -2213,13 +2340,36 @@
       <c r="J34" t="n">
         <v>11</v>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" s="10" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending. Listed under Bodinga in your email table, but this ward is registered under Gwadabawa in our records - please confirm.</t>
+        </is>
+      </c>
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2237,14 +2387,11 @@
           <t>Mammande</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
         <v>1</v>
       </c>
@@ -2254,13 +2401,36 @@
       <c r="J35" t="n">
         <v>6</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" s="10" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O35" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2278,7 +2448,6 @@
           <t>Sabon Birni</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2303,13 +2472,36 @@
       <c r="J36" t="n">
         <v>4</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" s="10" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O36" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2327,7 +2519,6 @@
           <t>Mamman Suka</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2352,13 +2543,36 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" s="10" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O37" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2376,14 +2590,11 @@
           <t>Gandi 1</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
         <v>4</v>
       </c>
@@ -2393,13 +2604,7 @@
       <c r="J38" t="n">
         <v>42</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" s="10" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2417,14 +2622,11 @@
           <t>Kurya</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
         <v>1</v>
       </c>
@@ -2434,13 +2636,7 @@
       <c r="J39" t="n">
         <v>42</v>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" s="10" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2458,14 +2654,11 @@
           <t>Goddodi</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
         <v>3</v>
       </c>
@@ -2475,13 +2668,7 @@
       <c r="J40" t="n">
         <v>30</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" s="10" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2499,7 +2686,6 @@
           <t>Rabah</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2524,13 +2710,7 @@
       <c r="J41" t="n">
         <v>30</v>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" s="10" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2548,14 +2728,11 @@
           <t>Maikujera</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
         <v>2</v>
       </c>
@@ -2565,13 +2742,7 @@
       <c r="J42" t="n">
         <v>12</v>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" s="10" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2589,14 +2760,11 @@
           <t>Yarstakuwa</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
         <v>2</v>
       </c>
@@ -2606,13 +2774,7 @@
       <c r="J43" t="n">
         <v>12</v>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" s="10" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2630,14 +2792,11 @@
           <t>Rarah</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
         <v>2</v>
       </c>
@@ -2647,13 +2806,7 @@
       <c r="J44" t="n">
         <v>10</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" s="10" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2671,7 +2824,6 @@
           <t>Tsamiya</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2696,13 +2848,7 @@
       <c r="J45" t="n">
         <v>8</v>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" s="10" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2720,14 +2866,11 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
         <v>1</v>
       </c>
@@ -2737,13 +2880,7 @@
       <c r="J46" t="n">
         <v>6</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" s="10" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2761,14 +2898,11 @@
           <t>Tofa</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
         <v>1</v>
       </c>
@@ -2778,13 +2912,7 @@
       <c r="J47" t="n">
         <v>6</v>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
       <c r="O47" s="10" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2802,14 +2930,11 @@
           <t>Gandi 2</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
         <v>1</v>
       </c>
@@ -2819,13 +2944,7 @@
       <c r="J48" t="n">
         <v>0</v>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
       <c r="O48" s="10" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2843,14 +2962,11 @@
           <t>Romo Sarki</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
         <v>2</v>
       </c>
@@ -2860,13 +2976,7 @@
       <c r="J49" t="n">
         <v>42</v>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
       <c r="O49" s="10" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2884,14 +2994,11 @@
           <t>Tambuwal</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
         <v>2</v>
       </c>
@@ -2901,13 +3008,36 @@
       <c r="J50" t="n">
         <v>36</v>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" s="10" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O50" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2925,7 +3055,6 @@
           <t>Jabo-Kagara</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2950,13 +3079,36 @@
       <c r="J51" t="n">
         <v>30</v>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" s="10" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O51" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2974,14 +3126,11 @@
           <t>Bagida</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
         <v>4</v>
       </c>
@@ -2991,13 +3140,7 @@
       <c r="J52" t="n">
         <v>21</v>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" s="10" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3015,14 +3158,11 @@
           <t>Barkeji-Nabaguda</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
         <v>2</v>
       </c>
@@ -3032,13 +3172,36 @@
       <c r="J53" t="n">
         <v>18</v>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" s="10" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending. Your email listed this as "Nabaguda" - matched to this ward, please confirm.</t>
+        </is>
+      </c>
+      <c r="O53" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3056,14 +3219,11 @@
           <t>Sanyinna</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
         <v>1</v>
       </c>
@@ -3073,13 +3233,7 @@
       <c r="J54" t="n">
         <v>18</v>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" s="10" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3097,14 +3251,11 @@
           <t>Saida Goshe</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
         <v>1</v>
       </c>
@@ -3114,13 +3265,7 @@
       <c r="J55" t="n">
         <v>12</v>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" s="10" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3138,14 +3283,11 @@
           <t>Faga Alasan</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
         <v>1</v>
       </c>
@@ -3155,13 +3297,7 @@
       <c r="J56" t="n">
         <v>10</v>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" s="10" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3179,14 +3315,11 @@
           <t>Bashire-Maikada</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
         <v>2</v>
       </c>
@@ -3196,13 +3329,36 @@
       <c r="J57" t="n">
         <v>8</v>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" s="10" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Insecurity / conflict</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O57" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3220,14 +3376,11 @@
           <t>Dogon Daji</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
         <v>1</v>
       </c>
@@ -3237,13 +3390,36 @@
       <c r="J58" t="n">
         <v>6</v>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" s="10" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>N/A - fully accessible</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Reported by ACF following the Joint MSNA refresher training (email, 2026-09-04) - part of a partial list, ACF's consolidated version (incl. STCI) still pending.</t>
+        </is>
+      </c>
+      <c r="O58" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3261,7 +3437,6 @@
           <t>Sabon Birni</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3286,13 +3461,7 @@
       <c r="J59" t="n">
         <v>3</v>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" s="10" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
+      <c r="O59" s="10" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -3464,13 +3633,7 @@
           <t>24</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" s="10" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3513,13 +3676,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" s="10" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3562,13 +3719,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" s="10" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3611,13 +3762,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" s="10" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3645,7 +3790,6 @@
           <t>non_idp_NG034002_1</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>6</t>
@@ -3656,13 +3800,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" s="10" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3690,7 +3828,6 @@
           <t>non_idp_NG034002_10</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>6</t>
@@ -3701,13 +3838,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3735,7 +3866,6 @@
           <t>non_idp_NG034002_11</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>6</t>
@@ -3746,13 +3876,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3780,7 +3904,6 @@
           <t>non_idp_NG034002_12</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>6</t>
@@ -3791,13 +3914,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3825,7 +3942,6 @@
           <t>non_idp_NG034002_13</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>6</t>
@@ -3836,13 +3952,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" s="10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3870,7 +3980,6 @@
           <t>non_idp_NG034002_14</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>6</t>
@@ -3881,13 +3990,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" s="10" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3915,7 +4018,6 @@
           <t>non_idp_NG034002_15</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>6</t>
@@ -3926,13 +4028,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" s="10" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3960,7 +4056,6 @@
           <t>non_idp_NG034002_16</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>6</t>
@@ -3971,13 +4066,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" s="10" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4005,7 +4094,6 @@
           <t>non_idp_NG034002_17</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>6</t>
@@ -4016,13 +4104,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" s="10" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4050,7 +4132,6 @@
           <t>non_idp_NG034002_2</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>6</t>
@@ -4061,13 +4142,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" s="10" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4095,7 +4170,6 @@
           <t>non_idp_NG034002_3</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>6</t>
@@ -4106,13 +4180,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" s="10" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4140,7 +4208,6 @@
           <t>non_idp_NG034002_4</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>6</t>
@@ -4151,13 +4218,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" s="10" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4185,7 +4246,6 @@
           <t>non_idp_NG034002_5</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>6</t>
@@ -4196,13 +4256,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" s="10" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4230,7 +4284,6 @@
           <t>non_idp_NG034002_6</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>6</t>
@@ -4241,13 +4294,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" s="10" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4275,7 +4322,6 @@
           <t>non_idp_NG034002_7</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>6</t>
@@ -4286,13 +4332,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" s="10" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4320,7 +4360,6 @@
           <t>non_idp_NG034002_8</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>6</t>
@@ -4331,13 +4370,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" s="10" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4365,7 +4398,6 @@
           <t>non_idp_NG034002_9</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>6</t>
@@ -4376,13 +4408,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" s="10" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4425,13 +4451,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" s="10" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4474,13 +4494,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" s="10" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4523,13 +4537,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" s="10" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4572,13 +4580,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" s="10" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4606,7 +4608,6 @@
           <t>non_idp_NG034006_1</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>6</t>
@@ -4617,13 +4618,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" s="10" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4651,7 +4646,6 @@
           <t>non_idp_NG034006_11</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>6</t>
@@ -4662,13 +4656,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" s="10" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4696,7 +4684,6 @@
           <t>non_idp_NG034006_12</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>6</t>
@@ -4707,13 +4694,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" s="10" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4741,7 +4722,6 @@
           <t>non_idp_NG034006_13</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>6</t>
@@ -4752,13 +4732,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" s="10" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4786,7 +4760,6 @@
           <t>non_idp_NG034006_14</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>6</t>
@@ -4797,13 +4770,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" s="10" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4831,7 +4798,6 @@
           <t>non_idp_NG034006_15</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>6</t>
@@ -4842,13 +4808,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" s="10" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4876,7 +4836,6 @@
           <t>non_idp_NG034006_16</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>6</t>
@@ -4887,13 +4846,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" s="10" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4921,7 +4874,6 @@
           <t>non_idp_NG034006_17</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>6</t>
@@ -4932,13 +4884,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" s="10" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4966,7 +4912,6 @@
           <t>non_idp_NG034006_2</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>6</t>
@@ -4977,13 +4922,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" s="10" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5011,7 +4950,6 @@
           <t>non_idp_NG034006_3</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>6</t>
@@ -5022,13 +4960,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" s="10" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5056,7 +4988,6 @@
           <t>non_idp_NG034006_4</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>6</t>
@@ -5067,13 +4998,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" s="10" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5101,7 +5026,6 @@
           <t>non_idp_NG034006_5</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>6</t>
@@ -5112,13 +5036,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" s="10" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5146,7 +5064,6 @@
           <t>non_idp_NG034006_6</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>6</t>
@@ -5157,13 +5074,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" s="10" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5191,7 +5102,6 @@
           <t>non_idp_NG034006_7</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>6</t>
@@ -5202,13 +5112,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" s="10" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5236,7 +5140,6 @@
           <t>non_idp_NG034006_8</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>6</t>
@@ -5247,13 +5150,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" s="10" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5281,7 +5178,6 @@
           <t>non_idp_NG034006_9</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>12</t>
@@ -5292,13 +5188,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" s="10" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5341,13 +5231,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" s="10" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5390,13 +5274,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" s="10" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5439,13 +5317,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" s="10" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5488,13 +5360,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" s="10" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5522,7 +5388,6 @@
           <t>non_idp_NG034005_1</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>6</t>
@@ -5533,13 +5398,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" s="10" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5567,7 +5426,6 @@
           <t>non_idp_NG034005_10</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>6</t>
@@ -5578,13 +5436,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" s="10" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5612,7 +5464,6 @@
           <t>non_idp_NG034005_11</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>6</t>
@@ -5623,13 +5474,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" s="10" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5657,7 +5502,6 @@
           <t>non_idp_NG034005_12</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>6</t>
@@ -5668,13 +5512,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
       <c r="M50" s="10" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5702,7 +5540,6 @@
           <t>non_idp_NG034005_13</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>6</t>
@@ -5713,13 +5550,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
       <c r="M51" s="10" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5747,7 +5578,6 @@
           <t>non_idp_NG034005_14</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>6</t>
@@ -5758,13 +5588,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
       <c r="M52" s="10" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5792,7 +5616,6 @@
           <t>non_idp_NG034005_15</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>6</t>
@@ -5803,13 +5626,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
       <c r="M53" s="10" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5837,7 +5654,6 @@
           <t>non_idp_NG034005_16</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>6</t>
@@ -5848,13 +5664,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" s="10" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5882,7 +5692,6 @@
           <t>non_idp_NG034005_17</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>6</t>
@@ -5893,13 +5702,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" s="10" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5927,7 +5730,6 @@
           <t>non_idp_NG034005_2</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>6</t>
@@ -5938,13 +5740,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" s="10" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5972,7 +5768,6 @@
           <t>non_idp_NG034005_3</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>6</t>
@@ -5983,13 +5778,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" s="10" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6017,7 +5806,6 @@
           <t>non_idp_NG034005_4</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>6</t>
@@ -6028,13 +5816,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" s="10" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6062,7 +5844,6 @@
           <t>non_idp_NG034005_5</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>6</t>
@@ -6073,13 +5854,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" s="10" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6107,7 +5882,6 @@
           <t>non_idp_NG034005_6</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>6</t>
@@ -6118,13 +5892,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" s="10" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6152,7 +5920,6 @@
           <t>non_idp_NG034005_7</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>6</t>
@@ -6163,13 +5930,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" s="10" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6197,7 +5958,6 @@
           <t>non_idp_NG034005_8</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>6</t>
@@ -6208,13 +5968,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" s="10" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6242,7 +5996,6 @@
           <t>non_idp_NG034005_9</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>6</t>
@@ -6253,13 +6006,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" s="10" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6302,13 +6049,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" s="10" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6351,13 +6092,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" s="10" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6400,13 +6135,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" s="10" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6449,13 +6178,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
       <c r="M67" s="10" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6483,7 +6206,6 @@
           <t>non_idp_NG034012_1</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>6</t>
@@ -6494,13 +6216,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
       <c r="M68" s="10" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6528,7 +6244,6 @@
           <t>non_idp_NG034012_10</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>6</t>
@@ -6539,13 +6254,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
       <c r="M69" s="10" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6573,7 +6282,6 @@
           <t>non_idp_NG034012_11</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>6</t>
@@ -6584,13 +6292,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
       <c r="M70" s="10" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6618,7 +6320,6 @@
           <t>non_idp_NG034012_12</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>6</t>
@@ -6629,13 +6330,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" s="10" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6663,7 +6358,6 @@
           <t>non_idp_NG034012_13</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>6</t>
@@ -6674,13 +6368,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" s="10" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6708,7 +6396,6 @@
           <t>non_idp_NG034012_14</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>6</t>
@@ -6719,13 +6406,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" s="10" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6753,7 +6434,6 @@
           <t>non_idp_NG034012_15</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>6</t>
@@ -6764,13 +6444,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" s="10" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6798,7 +6472,6 @@
           <t>non_idp_NG034012_16</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>6</t>
@@ -6809,13 +6482,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" s="10" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6843,7 +6510,6 @@
           <t>non_idp_NG034012_17</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>6</t>
@@ -6854,13 +6520,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" s="10" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6888,7 +6548,6 @@
           <t>non_idp_NG034012_2</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>6</t>
@@ -6899,13 +6558,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" s="10" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6933,7 +6586,6 @@
           <t>non_idp_NG034012_3</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>6</t>
@@ -6944,13 +6596,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" s="10" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6978,7 +6624,6 @@
           <t>non_idp_NG034012_4</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>6</t>
@@ -6989,13 +6634,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" s="10" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7023,7 +6662,6 @@
           <t>non_idp_NG034012_5</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>6</t>
@@ -7034,13 +6672,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" s="10" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7068,7 +6700,6 @@
           <t>non_idp_NG034012_6</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>6</t>
@@ -7079,13 +6710,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
       <c r="M81" s="10" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7113,7 +6738,6 @@
           <t>non_idp_NG034012_7</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>6</t>
@@ -7124,13 +6748,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" s="10" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7158,7 +6776,6 @@
           <t>non_idp_NG034012_8</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>6</t>
@@ -7169,13 +6786,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
       <c r="M83" s="10" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7203,7 +6814,6 @@
           <t>non_idp_NG034012_9</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>6</t>
@@ -7214,13 +6824,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
       <c r="M84" s="10" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7263,13 +6867,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
       <c r="M85" s="10" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7312,13 +6910,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" s="10" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7361,13 +6953,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" s="10" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7410,13 +6996,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
       <c r="M88" s="10" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7459,13 +7039,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
       <c r="M89" s="10" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7508,13 +7082,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" s="10" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7557,13 +7125,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" s="10" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7606,13 +7168,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" s="10" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7640,7 +7196,6 @@
           <t>non_idp_NG034018_1</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>6</t>
@@ -7651,13 +7206,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" s="10" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7685,7 +7234,6 @@
           <t>non_idp_NG034018_10</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>6</t>
@@ -7696,13 +7244,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" s="10" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7730,7 +7272,6 @@
           <t>non_idp_NG034018_11</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>6</t>
@@ -7741,13 +7282,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" s="10" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7775,7 +7310,6 @@
           <t>non_idp_NG034018_12</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>6</t>
@@ -7786,13 +7320,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" s="10" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7820,7 +7348,6 @@
           <t>non_idp_NG034018_13</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>6</t>
@@ -7831,13 +7358,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" s="10" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7865,7 +7386,6 @@
           <t>non_idp_NG034018_14</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>6</t>
@@ -7876,13 +7396,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
       <c r="M98" s="10" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7910,7 +7424,6 @@
           <t>non_idp_NG034018_15</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>6</t>
@@ -7921,13 +7434,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
       <c r="M99" s="10" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7955,7 +7462,6 @@
           <t>non_idp_NG034018_16</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>6</t>
@@ -7966,13 +7472,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
       <c r="M100" s="10" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8000,7 +7500,6 @@
           <t>non_idp_NG034018_17</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>6</t>
@@ -8011,13 +7510,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
       <c r="M101" s="10" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8045,7 +7538,6 @@
           <t>non_idp_NG034018_2</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>6</t>
@@ -8056,13 +7548,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
       <c r="M102" s="10" t="inlineStr"/>
-      <c r="N102" t="inlineStr"/>
-      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8090,7 +7576,6 @@
           <t>non_idp_NG034018_3</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>6</t>
@@ -8101,13 +7586,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
       <c r="M103" s="10" t="inlineStr"/>
-      <c r="N103" t="inlineStr"/>
-      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8135,7 +7614,6 @@
           <t>non_idp_NG034018_4</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>6</t>
@@ -8146,13 +7624,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
       <c r="M104" s="10" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
-      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8180,7 +7652,6 @@
           <t>non_idp_NG034018_5</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>6</t>
@@ -8191,13 +7662,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" s="10" t="inlineStr"/>
-      <c r="N105" t="inlineStr"/>
-      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8225,7 +7690,6 @@
           <t>non_idp_NG034018_6</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>12</t>
@@ -8236,13 +7700,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" s="10" t="inlineStr"/>
-      <c r="N106" t="inlineStr"/>
-      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8270,7 +7728,6 @@
           <t>non_idp_NG034018_8</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>6</t>
@@ -8281,13 +7738,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
       <c r="M107" s="10" t="inlineStr"/>
-      <c r="N107" t="inlineStr"/>
-      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8315,7 +7766,6 @@
           <t>non_idp_NG034018_9</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>6</t>
@@ -8326,13 +7776,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" s="10" t="inlineStr"/>
-      <c r="N108" t="inlineStr"/>
-      <c r="O108" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -8616,13 +8060,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{759D2E2A-1754-49D5-9966-704A7B9FBF6E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4F1B008-F475-4649-8995-8F32287A8344}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A21BC48-8A83-4CCE-86FA-71B1ACDF6EA9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1BBD728-8580-44F2-894E-A167B7A06FBA}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2FBA7F5-0CF1-4ADF-B98F-155A518A0073}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5F4F354-F89D-4892-BC58-E44E67F6CF23}"/>
 </file>
</xml_diff>